<commit_message>
Diseño ventana emergente OM
</commit_message>
<xml_diff>
--- a/data/raw/Plan de accion/PA_1.xlsx
+++ b/data/raw/Plan de accion/PA_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/Sistema_Indicadores_Poli/data/raw/Plan de accion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_C4BD844F18F46918874719FA9983E268DB8A1E7B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56C9A60F-6037-4FA0-9CFE-BBF97636A5E8}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_C4BD844F18F46918874719FA9983E268DB8A1E7B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{947BB957-97EC-4B3C-8E84-08056F005DD6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4323,7 +4323,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AE422"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4427,7 +4426,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
         <v>1141</v>
       </c>
@@ -4506,7 +4505,7 @@
       <c r="AD2" s="8"/>
       <c r="AE2" s="8"/>
     </row>
-    <row r="3" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>1142</v>
       </c>
@@ -4585,7 +4584,7 @@
       <c r="AD3" s="8"/>
       <c r="AE3" s="8"/>
     </row>
-    <row r="4" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>1244</v>
       </c>
@@ -4664,7 +4663,7 @@
       <c r="AD4" s="8"/>
       <c r="AE4" s="8"/>
     </row>
-    <row r="5" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>1280</v>
       </c>
@@ -4743,7 +4742,7 @@
       <c r="AD5" s="8"/>
       <c r="AE5" s="8"/>
     </row>
-    <row r="6" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>1285</v>
       </c>
@@ -4814,7 +4813,7 @@
       <c r="AD6" s="8"/>
       <c r="AE6" s="8"/>
     </row>
-    <row r="7" spans="1:31" ht="144" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:31" ht="144" x14ac:dyDescent="0.3">
       <c r="A7" s="8">
         <v>1292</v>
       </c>
@@ -4883,7 +4882,7 @@
       <c r="AD7" s="8"/>
       <c r="AE7" s="8"/>
     </row>
-    <row r="8" spans="1:31" ht="144" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:31" ht="144" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>1293</v>
       </c>
@@ -4952,7 +4951,7 @@
       <c r="AD8" s="8"/>
       <c r="AE8" s="8"/>
     </row>
-    <row r="9" spans="1:31" ht="144" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:31" ht="144" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>1294</v>
       </c>
@@ -5021,7 +5020,7 @@
       <c r="AD9" s="8"/>
       <c r="AE9" s="8"/>
     </row>
-    <row r="10" spans="1:31" ht="144" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" ht="144" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>1295</v>
       </c>
@@ -5090,7 +5089,7 @@
       <c r="AD10" s="8"/>
       <c r="AE10" s="8"/>
     </row>
-    <row r="11" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>1308</v>
       </c>
@@ -5167,7 +5166,7 @@
       <c r="AD11" s="8"/>
       <c r="AE11" s="8"/>
     </row>
-    <row r="12" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>1328</v>
       </c>
@@ -5246,7 +5245,7 @@
       <c r="AD12" s="8"/>
       <c r="AE12" s="8"/>
     </row>
-    <row r="13" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>1332</v>
       </c>
@@ -5313,7 +5312,7 @@
       <c r="AD13" s="8"/>
       <c r="AE13" s="8"/>
     </row>
-    <row r="14" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>1333</v>
       </c>
@@ -5380,7 +5379,7 @@
       <c r="AD14" s="8"/>
       <c r="AE14" s="8"/>
     </row>
-    <row r="15" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>1334</v>
       </c>
@@ -5447,7 +5446,7 @@
       <c r="AD15" s="8"/>
       <c r="AE15" s="8"/>
     </row>
-    <row r="16" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>1335</v>
       </c>
@@ -5514,7 +5513,7 @@
       <c r="AD16" s="8"/>
       <c r="AE16" s="8"/>
     </row>
-    <row r="17" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>1336</v>
       </c>
@@ -5587,7 +5586,7 @@
       <c r="AD17" s="8"/>
       <c r="AE17" s="8"/>
     </row>
-    <row r="18" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>1337</v>
       </c>
@@ -5658,7 +5657,7 @@
       <c r="AD18" s="8"/>
       <c r="AE18" s="8"/>
     </row>
-    <row r="19" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
         <v>1338</v>
       </c>
@@ -5729,7 +5728,7 @@
       <c r="AD19" s="8"/>
       <c r="AE19" s="8"/>
     </row>
-    <row r="20" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>1339</v>
       </c>
@@ -5808,7 +5807,7 @@
       <c r="AD20" s="8"/>
       <c r="AE20" s="8"/>
     </row>
-    <row r="21" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A21" s="8">
         <v>1340</v>
       </c>
@@ -5887,7 +5886,7 @@
       <c r="AD21" s="8"/>
       <c r="AE21" s="8"/>
     </row>
-    <row r="22" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A22" s="8">
         <v>1341</v>
       </c>
@@ -5966,7 +5965,7 @@
       <c r="AD22" s="8"/>
       <c r="AE22" s="8"/>
     </row>
-    <row r="23" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A23" s="8">
         <v>1342</v>
       </c>
@@ -6045,7 +6044,7 @@
       <c r="AD23" s="8"/>
       <c r="AE23" s="8"/>
     </row>
-    <row r="24" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A24" s="8">
         <v>1343</v>
       </c>
@@ -6124,7 +6123,7 @@
       <c r="AD24" s="8"/>
       <c r="AE24" s="8"/>
     </row>
-    <row r="25" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A25" s="8">
         <v>1344</v>
       </c>
@@ -6203,7 +6202,7 @@
       <c r="AD25" s="8"/>
       <c r="AE25" s="8"/>
     </row>
-    <row r="26" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A26" s="8">
         <v>1345</v>
       </c>
@@ -6282,7 +6281,7 @@
       <c r="AD26" s="8"/>
       <c r="AE26" s="8"/>
     </row>
-    <row r="27" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A27" s="8">
         <v>1346</v>
       </c>
@@ -6361,7 +6360,7 @@
       <c r="AD27" s="8"/>
       <c r="AE27" s="8"/>
     </row>
-    <row r="28" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A28" s="8">
         <v>1347</v>
       </c>
@@ -6440,7 +6439,7 @@
       <c r="AD28" s="8"/>
       <c r="AE28" s="8"/>
     </row>
-    <row r="29" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A29" s="8">
         <v>1348</v>
       </c>
@@ -6519,7 +6518,7 @@
       <c r="AD29" s="8"/>
       <c r="AE29" s="8"/>
     </row>
-    <row r="30" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A30" s="8">
         <v>1349</v>
       </c>
@@ -6598,7 +6597,7 @@
       <c r="AD30" s="8"/>
       <c r="AE30" s="8"/>
     </row>
-    <row r="31" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A31" s="8">
         <v>1350</v>
       </c>
@@ -6677,7 +6676,7 @@
       <c r="AD31" s="8"/>
       <c r="AE31" s="8"/>
     </row>
-    <row r="32" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A32" s="8">
         <v>1351</v>
       </c>
@@ -6756,7 +6755,7 @@
       <c r="AD32" s="8"/>
       <c r="AE32" s="8"/>
     </row>
-    <row r="33" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A33" s="8">
         <v>1353</v>
       </c>
@@ -6835,7 +6834,7 @@
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
     </row>
-    <row r="34" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A34" s="8">
         <v>1354</v>
       </c>
@@ -6914,7 +6913,7 @@
       <c r="AD34" s="8"/>
       <c r="AE34" s="8"/>
     </row>
-    <row r="35" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A35" s="8">
         <v>1355</v>
       </c>
@@ -6993,7 +6992,7 @@
       <c r="AD35" s="8"/>
       <c r="AE35" s="8"/>
     </row>
-    <row r="36" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A36" s="8">
         <v>1356</v>
       </c>
@@ -7072,7 +7071,7 @@
       <c r="AD36" s="8"/>
       <c r="AE36" s="8"/>
     </row>
-    <row r="37" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A37" s="8">
         <v>1357</v>
       </c>
@@ -7151,7 +7150,7 @@
       <c r="AD37" s="8"/>
       <c r="AE37" s="8"/>
     </row>
-    <row r="38" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A38" s="8">
         <v>1358</v>
       </c>
@@ -7230,7 +7229,7 @@
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
     </row>
-    <row r="39" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A39" s="8">
         <v>1359</v>
       </c>
@@ -7309,7 +7308,7 @@
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
     </row>
-    <row r="40" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A40" s="8">
         <v>1360</v>
       </c>
@@ -7388,7 +7387,7 @@
       <c r="AD40" s="8"/>
       <c r="AE40" s="8"/>
     </row>
-    <row r="41" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A41" s="8">
         <v>1361</v>
       </c>
@@ -7467,7 +7466,7 @@
       <c r="AD41" s="8"/>
       <c r="AE41" s="8"/>
     </row>
-    <row r="42" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A42" s="8">
         <v>1362</v>
       </c>
@@ -7546,7 +7545,7 @@
       <c r="AD42" s="8"/>
       <c r="AE42" s="8"/>
     </row>
-    <row r="43" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A43" s="8">
         <v>1363</v>
       </c>
@@ -7627,7 +7626,7 @@
       <c r="AD43" s="8"/>
       <c r="AE43" s="8"/>
     </row>
-    <row r="44" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A44" s="8">
         <v>1364</v>
       </c>
@@ -7706,7 +7705,7 @@
       <c r="AD44" s="8"/>
       <c r="AE44" s="8"/>
     </row>
-    <row r="45" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A45" s="8">
         <v>1365</v>
       </c>
@@ -7785,7 +7784,7 @@
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
     </row>
-    <row r="46" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A46" s="8">
         <v>1366</v>
       </c>
@@ -7866,7 +7865,7 @@
       <c r="AD46" s="8"/>
       <c r="AE46" s="8"/>
     </row>
-    <row r="47" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A47" s="8">
         <v>1367</v>
       </c>
@@ -7947,7 +7946,7 @@
       <c r="AD47" s="8"/>
       <c r="AE47" s="8"/>
     </row>
-    <row r="48" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A48" s="8">
         <v>1371</v>
       </c>
@@ -8026,7 +8025,7 @@
       <c r="AD48" s="8"/>
       <c r="AE48" s="8"/>
     </row>
-    <row r="49" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A49" s="8">
         <v>1375</v>
       </c>
@@ -8105,7 +8104,7 @@
       <c r="AD49" s="8"/>
       <c r="AE49" s="8"/>
     </row>
-    <row r="50" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A50" s="8">
         <v>1377</v>
       </c>
@@ -8184,7 +8183,7 @@
       <c r="AD50" s="8"/>
       <c r="AE50" s="8"/>
     </row>
-    <row r="51" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A51" s="8">
         <v>1378</v>
       </c>
@@ -8263,7 +8262,7 @@
       <c r="AD51" s="8"/>
       <c r="AE51" s="8"/>
     </row>
-    <row r="52" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A52" s="8">
         <v>1379</v>
       </c>
@@ -8340,7 +8339,7 @@
       <c r="AD52" s="8"/>
       <c r="AE52" s="8"/>
     </row>
-    <row r="53" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A53" s="8">
         <v>1382</v>
       </c>
@@ -8419,7 +8418,7 @@
       <c r="AD53" s="8"/>
       <c r="AE53" s="8"/>
     </row>
-    <row r="54" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A54" s="8">
         <v>1383</v>
       </c>
@@ -8498,7 +8497,7 @@
       <c r="AD54" s="8"/>
       <c r="AE54" s="8"/>
     </row>
-    <row r="55" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A55" s="8">
         <v>1395</v>
       </c>
@@ -8571,7 +8570,7 @@
       <c r="AD55" s="8"/>
       <c r="AE55" s="8"/>
     </row>
-    <row r="56" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A56" s="8">
         <v>1401</v>
       </c>
@@ -8644,7 +8643,7 @@
       <c r="AD56" s="8"/>
       <c r="AE56" s="8"/>
     </row>
-    <row r="57" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A57" s="8">
         <v>1405</v>
       </c>
@@ -8715,7 +8714,7 @@
       <c r="AD57" s="8"/>
       <c r="AE57" s="8"/>
     </row>
-    <row r="58" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A58" s="8">
         <v>1406</v>
       </c>
@@ -8788,7 +8787,7 @@
       <c r="AD58" s="8"/>
       <c r="AE58" s="8"/>
     </row>
-    <row r="59" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A59" s="8">
         <v>1413</v>
       </c>
@@ -8869,7 +8868,7 @@
       <c r="AD59" s="8"/>
       <c r="AE59" s="8"/>
     </row>
-    <row r="60" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A60" s="8">
         <v>1415</v>
       </c>
@@ -8950,7 +8949,7 @@
       <c r="AD60" s="8"/>
       <c r="AE60" s="8"/>
     </row>
-    <row r="61" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A61" s="8">
         <v>1433</v>
       </c>
@@ -9029,7 +9028,7 @@
       <c r="AD61" s="8"/>
       <c r="AE61" s="8"/>
     </row>
-    <row r="62" spans="1:31" ht="403.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:31" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A62" s="8">
         <v>1435</v>
       </c>
@@ -9104,7 +9103,7 @@
       <c r="AD62" s="8"/>
       <c r="AE62" s="8"/>
     </row>
-    <row r="63" spans="1:31" ht="403.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:31" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A63" s="8">
         <v>1436</v>
       </c>
@@ -9179,7 +9178,7 @@
       <c r="AD63" s="8"/>
       <c r="AE63" s="8"/>
     </row>
-    <row r="64" spans="1:31" ht="403.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:31" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A64" s="8">
         <v>1437</v>
       </c>
@@ -9254,7 +9253,7 @@
       <c r="AD64" s="8"/>
       <c r="AE64" s="8"/>
     </row>
-    <row r="65" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A65" s="8">
         <v>1438</v>
       </c>
@@ -9333,7 +9332,7 @@
       <c r="AD65" s="8"/>
       <c r="AE65" s="8"/>
     </row>
-    <row r="66" spans="1:31" ht="201.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:31" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A66" s="8">
         <v>1441</v>
       </c>
@@ -9406,7 +9405,7 @@
       <c r="AD66" s="8"/>
       <c r="AE66" s="8"/>
     </row>
-    <row r="67" spans="1:31" ht="201.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:31" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A67" s="8">
         <v>1442</v>
       </c>
@@ -9479,7 +9478,7 @@
       <c r="AD67" s="8"/>
       <c r="AE67" s="8"/>
     </row>
-    <row r="68" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A68" s="8">
         <v>1445</v>
       </c>
@@ -9554,7 +9553,7 @@
       <c r="AD68" s="8"/>
       <c r="AE68" s="8"/>
     </row>
-    <row r="69" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A69" s="8">
         <v>1446</v>
       </c>
@@ -9629,7 +9628,7 @@
       <c r="AD69" s="8"/>
       <c r="AE69" s="8"/>
     </row>
-    <row r="70" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A70" s="8">
         <v>1447</v>
       </c>
@@ -9704,7 +9703,7 @@
       <c r="AD70" s="8"/>
       <c r="AE70" s="8"/>
     </row>
-    <row r="71" spans="1:31" ht="158.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:31" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A71" s="8">
         <v>1468</v>
       </c>
@@ -9773,7 +9772,7 @@
       <c r="AD71" s="8"/>
       <c r="AE71" s="8"/>
     </row>
-    <row r="72" spans="1:31" ht="158.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:31" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A72" s="8">
         <v>1469</v>
       </c>
@@ -9842,7 +9841,7 @@
       <c r="AD72" s="8"/>
       <c r="AE72" s="8"/>
     </row>
-    <row r="73" spans="1:31" ht="158.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:31" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A73" s="8">
         <v>1470</v>
       </c>
@@ -9911,7 +9910,7 @@
       <c r="AD73" s="8"/>
       <c r="AE73" s="8"/>
     </row>
-    <row r="74" spans="1:31" ht="158.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:31" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A74" s="8">
         <v>1471</v>
       </c>
@@ -9980,7 +9979,7 @@
       <c r="AD74" s="8"/>
       <c r="AE74" s="8"/>
     </row>
-    <row r="75" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A75" s="8">
         <v>1476</v>
       </c>
@@ -10051,7 +10050,7 @@
       <c r="AD75" s="8"/>
       <c r="AE75" s="8"/>
     </row>
-    <row r="76" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A76" s="8">
         <v>1478</v>
       </c>
@@ -10130,7 +10129,7 @@
       <c r="AD76" s="8"/>
       <c r="AE76" s="8"/>
     </row>
-    <row r="77" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A77" s="8">
         <v>1479</v>
       </c>
@@ -10209,7 +10208,7 @@
       <c r="AD77" s="8"/>
       <c r="AE77" s="8"/>
     </row>
-    <row r="78" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A78" s="8">
         <v>1480</v>
       </c>
@@ -10288,7 +10287,7 @@
       <c r="AD78" s="8"/>
       <c r="AE78" s="8"/>
     </row>
-    <row r="79" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A79" s="8">
         <v>1481</v>
       </c>
@@ -10367,7 +10366,7 @@
       <c r="AD79" s="8"/>
       <c r="AE79" s="8"/>
     </row>
-    <row r="80" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A80" s="8">
         <v>1482</v>
       </c>
@@ -10448,7 +10447,7 @@
       <c r="AD80" s="8"/>
       <c r="AE80" s="8"/>
     </row>
-    <row r="81" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A81" s="8">
         <v>1483</v>
       </c>
@@ -10529,7 +10528,7 @@
       <c r="AD81" s="8"/>
       <c r="AE81" s="8"/>
     </row>
-    <row r="82" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A82" s="8">
         <v>1484</v>
       </c>
@@ -10610,7 +10609,7 @@
       <c r="AD82" s="8"/>
       <c r="AE82" s="8"/>
     </row>
-    <row r="83" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A83" s="8">
         <v>1485</v>
       </c>
@@ -10689,7 +10688,7 @@
       <c r="AD83" s="8"/>
       <c r="AE83" s="8"/>
     </row>
-    <row r="84" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A84" s="8">
         <v>1487</v>
       </c>
@@ -10756,7 +10755,7 @@
       <c r="AD84" s="8"/>
       <c r="AE84" s="8"/>
     </row>
-    <row r="85" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A85" s="8">
         <v>1489</v>
       </c>
@@ -10823,7 +10822,7 @@
       <c r="AD85" s="8"/>
       <c r="AE85" s="8"/>
     </row>
-    <row r="86" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A86" s="8">
         <v>1490</v>
       </c>
@@ -10902,7 +10901,7 @@
       <c r="AD86" s="8"/>
       <c r="AE86" s="8"/>
     </row>
-    <row r="87" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A87" s="8">
         <v>1491</v>
       </c>
@@ -10981,7 +10980,7 @@
       <c r="AD87" s="8"/>
       <c r="AE87" s="8"/>
     </row>
-    <row r="88" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A88" s="8">
         <v>1492</v>
       </c>
@@ -11060,7 +11059,7 @@
       <c r="AD88" s="8"/>
       <c r="AE88" s="8"/>
     </row>
-    <row r="89" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A89" s="8">
         <v>1493</v>
       </c>
@@ -11139,7 +11138,7 @@
       <c r="AD89" s="8"/>
       <c r="AE89" s="8"/>
     </row>
-    <row r="90" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A90" s="8">
         <v>1494</v>
       </c>
@@ -11218,7 +11217,7 @@
       <c r="AD90" s="8"/>
       <c r="AE90" s="8"/>
     </row>
-    <row r="91" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A91" s="8">
         <v>1495</v>
       </c>
@@ -11297,7 +11296,7 @@
       <c r="AD91" s="8"/>
       <c r="AE91" s="8"/>
     </row>
-    <row r="92" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A92" s="8">
         <v>1496</v>
       </c>
@@ -11376,7 +11375,7 @@
       <c r="AD92" s="8"/>
       <c r="AE92" s="8"/>
     </row>
-    <row r="93" spans="1:31" ht="216" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:31" ht="216" x14ac:dyDescent="0.3">
       <c r="A93" s="8">
         <v>1497</v>
       </c>
@@ -11455,7 +11454,7 @@
       <c r="AD93" s="8"/>
       <c r="AE93" s="8"/>
     </row>
-    <row r="94" spans="1:31" ht="273.60000000000002" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:31" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A94" s="8">
         <v>1498</v>
       </c>
@@ -11536,7 +11535,7 @@
       <c r="AD94" s="8"/>
       <c r="AE94" s="8"/>
     </row>
-    <row r="95" spans="1:31" ht="273.60000000000002" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:31" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A95" s="8">
         <v>1499</v>
       </c>
@@ -11617,7 +11616,7 @@
       <c r="AD95" s="8"/>
       <c r="AE95" s="8"/>
     </row>
-    <row r="96" spans="1:31" ht="273.60000000000002" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:31" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A96" s="8">
         <v>1500</v>
       </c>
@@ -11698,7 +11697,7 @@
       <c r="AD96" s="8"/>
       <c r="AE96" s="8"/>
     </row>
-    <row r="97" spans="1:31" ht="273.60000000000002" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:31" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A97" s="8">
         <v>1501</v>
       </c>
@@ -11777,7 +11776,7 @@
       <c r="AD97" s="8"/>
       <c r="AE97" s="8"/>
     </row>
-    <row r="98" spans="1:31" ht="244.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:31" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A98" s="8">
         <v>1504</v>
       </c>
@@ -11856,7 +11855,7 @@
       <c r="AD98" s="8"/>
       <c r="AE98" s="8"/>
     </row>
-    <row r="99" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A99" s="8">
         <v>1505</v>
       </c>
@@ -11935,7 +11934,7 @@
       <c r="AD99" s="8"/>
       <c r="AE99" s="8"/>
     </row>
-    <row r="100" spans="1:31" ht="244.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:31" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A100" s="8">
         <v>1506</v>
       </c>
@@ -12014,7 +12013,7 @@
       <c r="AD100" s="8"/>
       <c r="AE100" s="8"/>
     </row>
-    <row r="101" spans="1:31" ht="273.60000000000002" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:31" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A101" s="8">
         <v>1507</v>
       </c>
@@ -12091,7 +12090,7 @@
       <c r="AD101" s="8"/>
       <c r="AE101" s="8"/>
     </row>
-    <row r="102" spans="1:31" ht="273.60000000000002" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:31" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A102" s="8">
         <v>1508</v>
       </c>
@@ -12168,7 +12167,7 @@
       <c r="AD102" s="8"/>
       <c r="AE102" s="8"/>
     </row>
-    <row r="103" spans="1:31" ht="273.60000000000002" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:31" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A103" s="8">
         <v>1509</v>
       </c>
@@ -12245,7 +12244,7 @@
       <c r="AD103" s="8"/>
       <c r="AE103" s="8"/>
     </row>
-    <row r="104" spans="1:31" ht="273.60000000000002" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:31" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A104" s="8">
         <v>1510</v>
       </c>
@@ -12324,7 +12323,7 @@
       <c r="AD104" s="8"/>
       <c r="AE104" s="8"/>
     </row>
-    <row r="105" spans="1:31" ht="273.60000000000002" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:31" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A105" s="8">
         <v>1511</v>
       </c>
@@ -12401,7 +12400,7 @@
       <c r="AD105" s="8"/>
       <c r="AE105" s="8"/>
     </row>
-    <row r="106" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A106" s="8">
         <v>1512</v>
       </c>
@@ -12480,7 +12479,7 @@
       <c r="AD106" s="8"/>
       <c r="AE106" s="8"/>
     </row>
-    <row r="107" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A107" s="8">
         <v>1513</v>
       </c>
@@ -12561,7 +12560,7 @@
       <c r="AD107" s="8"/>
       <c r="AE107" s="8"/>
     </row>
-    <row r="108" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A108" s="8">
         <v>1515</v>
       </c>
@@ -12640,7 +12639,7 @@
       <c r="AD108" s="8"/>
       <c r="AE108" s="8"/>
     </row>
-    <row r="109" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A109" s="8">
         <v>1518</v>
       </c>
@@ -12719,7 +12718,7 @@
       <c r="AD109" s="8"/>
       <c r="AE109" s="8"/>
     </row>
-    <row r="110" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A110" s="8">
         <v>1519</v>
       </c>
@@ -12798,7 +12797,7 @@
       <c r="AD110" s="8"/>
       <c r="AE110" s="8"/>
     </row>
-    <row r="111" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A111" s="8">
         <v>1520</v>
       </c>
@@ -12877,7 +12876,7 @@
       <c r="AD111" s="8"/>
       <c r="AE111" s="8"/>
     </row>
-    <row r="112" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A112" s="8">
         <v>1521</v>
       </c>
@@ -12958,7 +12957,7 @@
       <c r="AD112" s="8"/>
       <c r="AE112" s="8"/>
     </row>
-    <row r="113" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A113" s="8">
         <v>1522</v>
       </c>
@@ -13039,7 +13038,7 @@
       <c r="AD113" s="8"/>
       <c r="AE113" s="8"/>
     </row>
-    <row r="114" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A114" s="8">
         <v>1523</v>
       </c>
@@ -13120,7 +13119,7 @@
       <c r="AD114" s="8"/>
       <c r="AE114" s="8"/>
     </row>
-    <row r="115" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A115" s="8">
         <v>1524</v>
       </c>
@@ -13201,7 +13200,7 @@
       <c r="AD115" s="8"/>
       <c r="AE115" s="8"/>
     </row>
-    <row r="116" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A116" s="8">
         <v>1525</v>
       </c>
@@ -13282,7 +13281,7 @@
       <c r="AD116" s="8"/>
       <c r="AE116" s="8"/>
     </row>
-    <row r="117" spans="1:31" ht="316.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:31" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A117" s="8">
         <v>1527</v>
       </c>
@@ -13363,7 +13362,7 @@
       <c r="AD117" s="8"/>
       <c r="AE117" s="8"/>
     </row>
-    <row r="118" spans="1:31" ht="316.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:31" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A118" s="8">
         <v>1529</v>
       </c>
@@ -13444,7 +13443,7 @@
       <c r="AD118" s="8"/>
       <c r="AE118" s="8"/>
     </row>
-    <row r="119" spans="1:31" ht="316.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:31" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A119" s="8">
         <v>1530</v>
       </c>
@@ -13525,7 +13524,7 @@
       <c r="AD119" s="8"/>
       <c r="AE119" s="8"/>
     </row>
-    <row r="120" spans="1:31" ht="316.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:31" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A120" s="8">
         <v>1531</v>
       </c>
@@ -13606,7 +13605,7 @@
       <c r="AD120" s="8"/>
       <c r="AE120" s="8"/>
     </row>
-    <row r="121" spans="1:31" ht="316.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:31" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A121" s="8">
         <v>1532</v>
       </c>
@@ -13687,7 +13686,7 @@
       <c r="AD121" s="8"/>
       <c r="AE121" s="8"/>
     </row>
-    <row r="122" spans="1:31" ht="316.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:31" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A122" s="8">
         <v>1533</v>
       </c>
@@ -13768,7 +13767,7 @@
       <c r="AD122" s="8"/>
       <c r="AE122" s="8"/>
     </row>
-    <row r="123" spans="1:31" ht="316.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:31" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A123" s="8">
         <v>1534</v>
       </c>
@@ -13849,7 +13848,7 @@
       <c r="AD123" s="8"/>
       <c r="AE123" s="8"/>
     </row>
-    <row r="124" spans="1:31" ht="316.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:31" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A124" s="8">
         <v>1535</v>
       </c>
@@ -13930,7 +13929,7 @@
       <c r="AD124" s="8"/>
       <c r="AE124" s="8"/>
     </row>
-    <row r="125" spans="1:31" ht="316.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:31" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A125" s="8">
         <v>1536</v>
       </c>
@@ -14011,7 +14010,7 @@
       <c r="AD125" s="8"/>
       <c r="AE125" s="8"/>
     </row>
-    <row r="126" spans="1:31" ht="316.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:31" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A126" s="8">
         <v>1537</v>
       </c>
@@ -14090,7 +14089,7 @@
       <c r="AD126" s="8"/>
       <c r="AE126" s="8"/>
     </row>
-    <row r="127" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A127" s="8">
         <v>1538</v>
       </c>
@@ -14163,7 +14162,7 @@
       <c r="AD127" s="8"/>
       <c r="AE127" s="8"/>
     </row>
-    <row r="128" spans="1:31" ht="374.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:31" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A128" s="8">
         <v>1541</v>
       </c>
@@ -14236,7 +14235,7 @@
       <c r="AD128" s="8"/>
       <c r="AE128" s="8"/>
     </row>
-    <row r="129" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A129" s="8">
         <v>1542</v>
       </c>
@@ -14309,7 +14308,7 @@
       <c r="AD129" s="8"/>
       <c r="AE129" s="8"/>
     </row>
-    <row r="130" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A130" s="8">
         <v>1543</v>
       </c>
@@ -14382,7 +14381,7 @@
       <c r="AD130" s="8"/>
       <c r="AE130" s="8"/>
     </row>
-    <row r="131" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A131" s="8">
         <v>1546</v>
       </c>
@@ -14455,7 +14454,7 @@
       <c r="AD131" s="8"/>
       <c r="AE131" s="8"/>
     </row>
-    <row r="132" spans="1:31" ht="201.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:31" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A132" s="8">
         <v>1549</v>
       </c>
@@ -14528,7 +14527,7 @@
       <c r="AD132" s="8"/>
       <c r="AE132" s="8"/>
     </row>
-    <row r="133" spans="1:31" ht="201.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:31" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A133" s="8">
         <v>1550</v>
       </c>
@@ -14601,7 +14600,7 @@
       <c r="AD133" s="8"/>
       <c r="AE133" s="8"/>
     </row>
-    <row r="134" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A134" s="8">
         <v>1551</v>
       </c>
@@ -14674,7 +14673,7 @@
       <c r="AD134" s="8"/>
       <c r="AE134" s="8"/>
     </row>
-    <row r="135" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A135" s="8">
         <v>1552</v>
       </c>
@@ -14747,7 +14746,7 @@
       <c r="AD135" s="8"/>
       <c r="AE135" s="8"/>
     </row>
-    <row r="136" spans="1:31" ht="345.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:31" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A136" s="8">
         <v>1555</v>
       </c>
@@ -14820,7 +14819,7 @@
       <c r="AD136" s="8"/>
       <c r="AE136" s="8"/>
     </row>
-    <row r="137" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A137" s="8">
         <v>1558</v>
       </c>
@@ -14893,7 +14892,7 @@
       <c r="AD137" s="8"/>
       <c r="AE137" s="8"/>
     </row>
-    <row r="138" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A138" s="8">
         <v>1559</v>
       </c>
@@ -14968,7 +14967,7 @@
       <c r="AD138" s="8"/>
       <c r="AE138" s="8"/>
     </row>
-    <row r="139" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A139" s="8">
         <v>1560</v>
       </c>
@@ -15045,7 +15044,7 @@
       <c r="AD139" s="8"/>
       <c r="AE139" s="8"/>
     </row>
-    <row r="140" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A140" s="8">
         <v>1561</v>
       </c>
@@ -15122,7 +15121,7 @@
       <c r="AD140" s="8"/>
       <c r="AE140" s="8"/>
     </row>
-    <row r="141" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A141" s="8">
         <v>1562</v>
       </c>
@@ -15199,7 +15198,7 @@
       <c r="AD141" s="8"/>
       <c r="AE141" s="8"/>
     </row>
-    <row r="142" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A142" s="8">
         <v>1563</v>
       </c>
@@ -15276,7 +15275,7 @@
       <c r="AD142" s="8"/>
       <c r="AE142" s="8"/>
     </row>
-    <row r="143" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A143" s="8">
         <v>1564</v>
       </c>
@@ -15353,7 +15352,7 @@
       <c r="AD143" s="8"/>
       <c r="AE143" s="8"/>
     </row>
-    <row r="144" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A144" s="8">
         <v>1565</v>
       </c>
@@ -15430,7 +15429,7 @@
       <c r="AD144" s="8"/>
       <c r="AE144" s="8"/>
     </row>
-    <row r="145" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A145" s="8">
         <v>1566</v>
       </c>
@@ -15507,7 +15506,7 @@
       <c r="AD145" s="8"/>
       <c r="AE145" s="8"/>
     </row>
-    <row r="146" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A146" s="8">
         <v>1567</v>
       </c>
@@ -15584,7 +15583,7 @@
       <c r="AD146" s="8"/>
       <c r="AE146" s="8"/>
     </row>
-    <row r="147" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A147" s="8">
         <v>1569</v>
       </c>
@@ -15659,7 +15658,7 @@
       <c r="AD147" s="8"/>
       <c r="AE147" s="8"/>
     </row>
-    <row r="148" spans="1:31" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:31" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A148" s="8">
         <v>1572</v>
       </c>
@@ -15736,7 +15735,7 @@
       <c r="AD148" s="8"/>
       <c r="AE148" s="8"/>
     </row>
-    <row r="149" spans="1:31" ht="374.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:31" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A149" s="8">
         <v>1573</v>
       </c>
@@ -15809,7 +15808,7 @@
       <c r="AD149" s="8"/>
       <c r="AE149" s="8"/>
     </row>
-    <row r="150" spans="1:31" ht="374.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:31" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A150" s="8">
         <v>1576</v>
       </c>
@@ -15882,7 +15881,7 @@
       <c r="AD150" s="8"/>
       <c r="AE150" s="8"/>
     </row>
-    <row r="151" spans="1:31" ht="374.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:31" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A151" s="8">
         <v>1577</v>
       </c>
@@ -15955,7 +15954,7 @@
       <c r="AD151" s="8"/>
       <c r="AE151" s="8"/>
     </row>
-    <row r="152" spans="1:31" ht="374.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:31" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A152" s="8">
         <v>1580</v>
       </c>
@@ -16028,7 +16027,7 @@
       <c r="AD152" s="8"/>
       <c r="AE152" s="8"/>
     </row>
-    <row r="153" spans="1:31" ht="374.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:31" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A153" s="8">
         <v>1581</v>
       </c>
@@ -16101,7 +16100,7 @@
       <c r="AD153" s="8"/>
       <c r="AE153" s="8"/>
     </row>
-    <row r="154" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A154" s="8">
         <v>1586</v>
       </c>
@@ -16170,7 +16169,7 @@
       <c r="AD154" s="8"/>
       <c r="AE154" s="8"/>
     </row>
-    <row r="155" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A155" s="8">
         <v>1587</v>
       </c>
@@ -16239,7 +16238,7 @@
       <c r="AD155" s="8"/>
       <c r="AE155" s="8"/>
     </row>
-    <row r="156" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A156" s="8">
         <v>1589</v>
       </c>
@@ -16308,7 +16307,7 @@
       <c r="AD156" s="8"/>
       <c r="AE156" s="8"/>
     </row>
-    <row r="157" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A157" s="8">
         <v>1590</v>
       </c>
@@ -16377,7 +16376,7 @@
       <c r="AD157" s="8"/>
       <c r="AE157" s="8"/>
     </row>
-    <row r="158" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A158" s="8">
         <v>1591</v>
       </c>
@@ -16448,7 +16447,7 @@
       <c r="AD158" s="8"/>
       <c r="AE158" s="8"/>
     </row>
-    <row r="159" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A159" s="8">
         <v>1592</v>
       </c>
@@ -16521,7 +16520,7 @@
       <c r="AD159" s="8"/>
       <c r="AE159" s="8"/>
     </row>
-    <row r="160" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A160" s="8">
         <v>1593</v>
       </c>
@@ -16594,7 +16593,7 @@
       <c r="AD160" s="8"/>
       <c r="AE160" s="8"/>
     </row>
-    <row r="161" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A161" s="8">
         <v>1594</v>
       </c>
@@ -16667,7 +16666,7 @@
       <c r="AD161" s="8"/>
       <c r="AE161" s="8"/>
     </row>
-    <row r="162" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A162" s="8">
         <v>1595</v>
       </c>
@@ -16748,7 +16747,7 @@
       <c r="AD162" s="8"/>
       <c r="AE162" s="8"/>
     </row>
-    <row r="163" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A163" s="8">
         <v>1596</v>
       </c>
@@ -16829,7 +16828,7 @@
       <c r="AD163" s="8"/>
       <c r="AE163" s="8"/>
     </row>
-    <row r="164" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A164" s="8">
         <v>1597</v>
       </c>
@@ -16910,7 +16909,7 @@
       <c r="AD164" s="8"/>
       <c r="AE164" s="8"/>
     </row>
-    <row r="165" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A165" s="8">
         <v>1598</v>
       </c>
@@ -16991,7 +16990,7 @@
       <c r="AD165" s="8"/>
       <c r="AE165" s="8"/>
     </row>
-    <row r="166" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A166" s="8">
         <v>1599</v>
       </c>
@@ -17072,7 +17071,7 @@
       <c r="AD166" s="8"/>
       <c r="AE166" s="8"/>
     </row>
-    <row r="167" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A167" s="8">
         <v>1600</v>
       </c>
@@ -17145,7 +17144,7 @@
       <c r="AD167" s="8"/>
       <c r="AE167" s="8"/>
     </row>
-    <row r="168" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A168" s="8">
         <v>1601</v>
       </c>
@@ -17218,7 +17217,7 @@
       <c r="AD168" s="8"/>
       <c r="AE168" s="8"/>
     </row>
-    <row r="169" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A169" s="8">
         <v>1602</v>
       </c>
@@ -17285,7 +17284,7 @@
       <c r="AD169" s="8"/>
       <c r="AE169" s="8"/>
     </row>
-    <row r="170" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A170" s="8">
         <v>1603</v>
       </c>
@@ -17368,7 +17367,7 @@
       <c r="AD170" s="8"/>
       <c r="AE170" s="8"/>
     </row>
-    <row r="171" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A171" s="8">
         <v>1604</v>
       </c>
@@ -17451,7 +17450,7 @@
       <c r="AD171" s="8"/>
       <c r="AE171" s="8"/>
     </row>
-    <row r="172" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A172" s="8">
         <v>1605</v>
       </c>
@@ -17534,7 +17533,7 @@
       <c r="AD172" s="8"/>
       <c r="AE172" s="8"/>
     </row>
-    <row r="173" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A173" s="8">
         <v>1606</v>
       </c>
@@ -17619,7 +17618,7 @@
       <c r="AD173" s="8"/>
       <c r="AE173" s="8"/>
     </row>
-    <row r="174" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A174" s="8">
         <v>1607</v>
       </c>
@@ -17704,7 +17703,7 @@
       <c r="AD174" s="8"/>
       <c r="AE174" s="8"/>
     </row>
-    <row r="175" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A175" s="8">
         <v>1608</v>
       </c>
@@ -17775,7 +17774,7 @@
       <c r="AD175" s="8"/>
       <c r="AE175" s="8"/>
     </row>
-    <row r="176" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A176" s="8">
         <v>1609</v>
       </c>
@@ -17846,7 +17845,7 @@
       <c r="AD176" s="8"/>
       <c r="AE176" s="8"/>
     </row>
-    <row r="177" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A177" s="8">
         <v>1610</v>
       </c>
@@ -17917,7 +17916,7 @@
       <c r="AD177" s="8"/>
       <c r="AE177" s="8"/>
     </row>
-    <row r="178" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A178" s="8">
         <v>1611</v>
       </c>
@@ -17988,7 +17987,7 @@
       <c r="AD178" s="8"/>
       <c r="AE178" s="8"/>
     </row>
-    <row r="179" spans="1:31" ht="259.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:31" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A179" s="8">
         <v>1612</v>
       </c>
@@ -18055,7 +18054,7 @@
       <c r="AD179" s="8"/>
       <c r="AE179" s="8"/>
     </row>
-    <row r="180" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A180" s="8">
         <v>1614</v>
       </c>
@@ -18136,7 +18135,7 @@
       <c r="AD180" s="8"/>
       <c r="AE180" s="8"/>
     </row>
-    <row r="181" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A181" s="8">
         <v>1615</v>
       </c>
@@ -18217,7 +18216,7 @@
       <c r="AD181" s="8"/>
       <c r="AE181" s="8"/>
     </row>
-    <row r="182" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A182" s="8">
         <v>1616</v>
       </c>
@@ -18298,7 +18297,7 @@
       <c r="AD182" s="8"/>
       <c r="AE182" s="8"/>
     </row>
-    <row r="183" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A183" s="8">
         <v>1617</v>
       </c>
@@ -18379,7 +18378,7 @@
       <c r="AD183" s="8"/>
       <c r="AE183" s="8"/>
     </row>
-    <row r="184" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A184" s="8">
         <v>1618</v>
       </c>
@@ -18460,7 +18459,7 @@
       <c r="AD184" s="8"/>
       <c r="AE184" s="8"/>
     </row>
-    <row r="185" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A185" s="8">
         <v>1621</v>
       </c>
@@ -18541,7 +18540,7 @@
       <c r="AD185" s="8"/>
       <c r="AE185" s="8"/>
     </row>
-    <row r="186" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A186" s="8">
         <v>1622</v>
       </c>
@@ -18622,7 +18621,7 @@
       <c r="AD186" s="8"/>
       <c r="AE186" s="8"/>
     </row>
-    <row r="187" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A187" s="8">
         <v>1623</v>
       </c>
@@ -18703,7 +18702,7 @@
       <c r="AD187" s="8"/>
       <c r="AE187" s="8"/>
     </row>
-    <row r="188" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A188" s="8">
         <v>1624</v>
       </c>
@@ -18784,7 +18783,7 @@
       <c r="AD188" s="8"/>
       <c r="AE188" s="8"/>
     </row>
-    <row r="189" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A189" s="8">
         <v>1625</v>
       </c>
@@ -18865,7 +18864,7 @@
       <c r="AD189" s="8"/>
       <c r="AE189" s="8"/>
     </row>
-    <row r="190" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A190" s="8">
         <v>1627</v>
       </c>
@@ -18936,7 +18935,7 @@
       <c r="AD190" s="8"/>
       <c r="AE190" s="8"/>
     </row>
-    <row r="191" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A191" s="8">
         <v>1628</v>
       </c>
@@ -19007,7 +19006,7 @@
       <c r="AD191" s="8"/>
       <c r="AE191" s="8"/>
     </row>
-    <row r="192" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A192" s="8">
         <v>1629</v>
       </c>
@@ -19078,7 +19077,7 @@
       <c r="AD192" s="8"/>
       <c r="AE192" s="8"/>
     </row>
-    <row r="193" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A193" s="8">
         <v>1630</v>
       </c>
@@ -19149,7 +19148,7 @@
       <c r="AD193" s="8"/>
       <c r="AE193" s="8"/>
     </row>
-    <row r="194" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A194" s="8">
         <v>1631</v>
       </c>
@@ -19216,7 +19215,7 @@
       <c r="AD194" s="8"/>
       <c r="AE194" s="8"/>
     </row>
-    <row r="195" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A195" s="8">
         <v>1632</v>
       </c>
@@ -19297,7 +19296,7 @@
       <c r="AD195" s="8"/>
       <c r="AE195" s="8"/>
     </row>
-    <row r="196" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A196" s="8">
         <v>1633</v>
       </c>
@@ -19378,7 +19377,7 @@
       <c r="AD196" s="8"/>
       <c r="AE196" s="8"/>
     </row>
-    <row r="197" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A197" s="8">
         <v>1634</v>
       </c>
@@ -19459,7 +19458,7 @@
       <c r="AD197" s="8"/>
       <c r="AE197" s="8"/>
     </row>
-    <row r="198" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A198" s="8">
         <v>1635</v>
       </c>
@@ -19540,7 +19539,7 @@
       <c r="AD198" s="8"/>
       <c r="AE198" s="8"/>
     </row>
-    <row r="199" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A199" s="8">
         <v>1636</v>
       </c>
@@ -19623,7 +19622,7 @@
       <c r="AD199" s="8"/>
       <c r="AE199" s="8"/>
     </row>
-    <row r="200" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A200" s="8">
         <v>1640</v>
       </c>
@@ -19702,7 +19701,7 @@
       <c r="AD200" s="8"/>
       <c r="AE200" s="8"/>
     </row>
-    <row r="201" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A201" s="8">
         <v>1641</v>
       </c>
@@ -19781,7 +19780,7 @@
       <c r="AD201" s="8"/>
       <c r="AE201" s="8"/>
     </row>
-    <row r="202" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A202" s="8">
         <v>1642</v>
       </c>
@@ -19860,7 +19859,7 @@
       <c r="AD202" s="8"/>
       <c r="AE202" s="8"/>
     </row>
-    <row r="203" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A203" s="8">
         <v>1643</v>
       </c>
@@ -19937,7 +19936,7 @@
       <c r="AD203" s="8"/>
       <c r="AE203" s="8"/>
     </row>
-    <row r="204" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A204" s="8">
         <v>1644</v>
       </c>
@@ -20014,7 +20013,7 @@
       <c r="AD204" s="8"/>
       <c r="AE204" s="8"/>
     </row>
-    <row r="205" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A205" s="8">
         <v>1645</v>
       </c>
@@ -20089,7 +20088,7 @@
       <c r="AD205" s="8"/>
       <c r="AE205" s="8"/>
     </row>
-    <row r="206" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A206" s="8">
         <v>1646</v>
       </c>
@@ -20164,7 +20163,7 @@
       <c r="AD206" s="8"/>
       <c r="AE206" s="8"/>
     </row>
-    <row r="207" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A207" s="8">
         <v>1647</v>
       </c>
@@ -20239,7 +20238,7 @@
       <c r="AD207" s="8"/>
       <c r="AE207" s="8"/>
     </row>
-    <row r="208" spans="1:31" ht="244.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:31" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A208" s="8">
         <v>1648</v>
       </c>
@@ -20314,7 +20313,7 @@
       <c r="AD208" s="8"/>
       <c r="AE208" s="8"/>
     </row>
-    <row r="209" spans="1:31" ht="244.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:31" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A209" s="8">
         <v>1649</v>
       </c>
@@ -20389,7 +20388,7 @@
       <c r="AD209" s="8"/>
       <c r="AE209" s="8"/>
     </row>
-    <row r="210" spans="1:31" ht="244.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:31" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A210" s="8">
         <v>1650</v>
       </c>
@@ -20464,7 +20463,7 @@
       <c r="AD210" s="8"/>
       <c r="AE210" s="8"/>
     </row>
-    <row r="211" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A211" s="8">
         <v>1653</v>
       </c>
@@ -20533,7 +20532,7 @@
       <c r="AD211" s="8"/>
       <c r="AE211" s="8"/>
     </row>
-    <row r="212" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A212" s="8">
         <v>1654</v>
       </c>
@@ -20602,7 +20601,7 @@
       <c r="AD212" s="8"/>
       <c r="AE212" s="8"/>
     </row>
-    <row r="213" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A213" s="8">
         <v>1655</v>
       </c>
@@ -20673,7 +20672,7 @@
       <c r="AD213" s="8"/>
       <c r="AE213" s="8"/>
     </row>
-    <row r="214" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A214" s="8">
         <v>1656</v>
       </c>
@@ -20744,7 +20743,7 @@
       <c r="AD214" s="8"/>
       <c r="AE214" s="8"/>
     </row>
-    <row r="215" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A215" s="8">
         <v>1657</v>
       </c>
@@ -20811,7 +20810,7 @@
       <c r="AD215" s="8"/>
       <c r="AE215" s="8"/>
     </row>
-    <row r="216" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A216" s="8">
         <v>1658</v>
       </c>
@@ -20882,7 +20881,7 @@
       <c r="AD216" s="8"/>
       <c r="AE216" s="8"/>
     </row>
-    <row r="217" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A217" s="8">
         <v>1659</v>
       </c>
@@ -20953,7 +20952,7 @@
       <c r="AD217" s="8"/>
       <c r="AE217" s="8"/>
     </row>
-    <row r="218" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A218" s="8">
         <v>1660</v>
       </c>
@@ -21022,7 +21021,7 @@
       <c r="AD218" s="8"/>
       <c r="AE218" s="8"/>
     </row>
-    <row r="219" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A219" s="8">
         <v>1661</v>
       </c>
@@ -21091,7 +21090,7 @@
       <c r="AD219" s="8"/>
       <c r="AE219" s="8"/>
     </row>
-    <row r="220" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A220" s="8">
         <v>1662</v>
       </c>
@@ -21160,7 +21159,7 @@
       <c r="AD220" s="8"/>
       <c r="AE220" s="8"/>
     </row>
-    <row r="221" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A221" s="8">
         <v>1663</v>
       </c>
@@ -21227,7 +21226,7 @@
       <c r="AD221" s="8"/>
       <c r="AE221" s="8"/>
     </row>
-    <row r="222" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A222" s="8">
         <v>1664</v>
       </c>
@@ -21296,7 +21295,7 @@
       <c r="AD222" s="8"/>
       <c r="AE222" s="8"/>
     </row>
-    <row r="223" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A223" s="8">
         <v>1665</v>
       </c>
@@ -21363,7 +21362,7 @@
       <c r="AD223" s="8"/>
       <c r="AE223" s="8"/>
     </row>
-    <row r="224" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A224" s="8">
         <v>1666</v>
       </c>
@@ -21434,7 +21433,7 @@
       <c r="AD224" s="8"/>
       <c r="AE224" s="8"/>
     </row>
-    <row r="225" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A225" s="8">
         <v>1667</v>
       </c>
@@ -21505,7 +21504,7 @@
       <c r="AD225" s="8"/>
       <c r="AE225" s="8"/>
     </row>
-    <row r="226" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A226" s="8">
         <v>1668</v>
       </c>
@@ -21572,7 +21571,7 @@
       <c r="AD226" s="8"/>
       <c r="AE226" s="8"/>
     </row>
-    <row r="227" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A227" s="8">
         <v>1671</v>
       </c>
@@ -21653,7 +21652,7 @@
       <c r="AD227" s="8"/>
       <c r="AE227" s="8"/>
     </row>
-    <row r="228" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A228" s="8">
         <v>1672</v>
       </c>
@@ -21734,7 +21733,7 @@
       <c r="AD228" s="8"/>
       <c r="AE228" s="8"/>
     </row>
-    <row r="229" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A229" s="8">
         <v>1673</v>
       </c>
@@ -21815,7 +21814,7 @@
       <c r="AD229" s="8"/>
       <c r="AE229" s="8"/>
     </row>
-    <row r="230" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A230" s="8">
         <v>1674</v>
       </c>
@@ -21896,7 +21895,7 @@
       <c r="AD230" s="8"/>
       <c r="AE230" s="8"/>
     </row>
-    <row r="231" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A231" s="8">
         <v>1675</v>
       </c>
@@ -21977,7 +21976,7 @@
       <c r="AD231" s="8"/>
       <c r="AE231" s="8"/>
     </row>
-    <row r="232" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A232" s="8">
         <v>1677</v>
       </c>
@@ -22058,7 +22057,7 @@
       <c r="AD232" s="8"/>
       <c r="AE232" s="8"/>
     </row>
-    <row r="233" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A233" s="8">
         <v>1678</v>
       </c>
@@ -22139,7 +22138,7 @@
       <c r="AD233" s="8"/>
       <c r="AE233" s="8"/>
     </row>
-    <row r="234" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A234" s="8">
         <v>1679</v>
       </c>
@@ -22220,7 +22219,7 @@
       <c r="AD234" s="8"/>
       <c r="AE234" s="8"/>
     </row>
-    <row r="235" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A235" s="8">
         <v>1680</v>
       </c>
@@ -22301,7 +22300,7 @@
       <c r="AD235" s="8"/>
       <c r="AE235" s="8"/>
     </row>
-    <row r="236" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A236" s="8">
         <v>1682</v>
       </c>
@@ -22372,7 +22371,7 @@
       <c r="AD236" s="8"/>
       <c r="AE236" s="8"/>
     </row>
-    <row r="237" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A237" s="8">
         <v>1683</v>
       </c>
@@ -22443,7 +22442,7 @@
       <c r="AD237" s="8"/>
       <c r="AE237" s="8"/>
     </row>
-    <row r="238" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A238" s="8">
         <v>1684</v>
       </c>
@@ -22514,7 +22513,7 @@
       <c r="AD238" s="8"/>
       <c r="AE238" s="8"/>
     </row>
-    <row r="239" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A239" s="8">
         <v>1685</v>
       </c>
@@ -22581,7 +22580,7 @@
       <c r="AD239" s="8"/>
       <c r="AE239" s="8"/>
     </row>
-    <row r="240" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A240" s="8">
         <v>1686</v>
       </c>
@@ -22648,7 +22647,7 @@
       <c r="AD240" s="8"/>
       <c r="AE240" s="8"/>
     </row>
-    <row r="241" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A241" s="8">
         <v>1688</v>
       </c>
@@ -22727,7 +22726,7 @@
       <c r="AD241" s="8"/>
       <c r="AE241" s="8"/>
     </row>
-    <row r="242" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A242" s="8">
         <v>1689</v>
       </c>
@@ -22806,7 +22805,7 @@
       <c r="AD242" s="8"/>
       <c r="AE242" s="8"/>
     </row>
-    <row r="243" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A243" s="8">
         <v>1690</v>
       </c>
@@ -22885,7 +22884,7 @@
       <c r="AD243" s="8"/>
       <c r="AE243" s="8"/>
     </row>
-    <row r="244" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A244" s="8">
         <v>1691</v>
       </c>
@@ -22964,7 +22963,7 @@
       <c r="AD244" s="8"/>
       <c r="AE244" s="8"/>
     </row>
-    <row r="245" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A245" s="8">
         <v>1692</v>
       </c>
@@ -23043,7 +23042,7 @@
       <c r="AD245" s="8"/>
       <c r="AE245" s="8"/>
     </row>
-    <row r="246" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A246" s="8">
         <v>1693</v>
       </c>
@@ -23114,7 +23113,7 @@
       <c r="AD246" s="8"/>
       <c r="AE246" s="8"/>
     </row>
-    <row r="247" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A247" s="8">
         <v>1694</v>
       </c>
@@ -23183,7 +23182,7 @@
       <c r="AD247" s="8"/>
       <c r="AE247" s="8"/>
     </row>
-    <row r="248" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A248" s="8">
         <v>1695</v>
       </c>
@@ -23254,7 +23253,7 @@
       <c r="AD248" s="8"/>
       <c r="AE248" s="8"/>
     </row>
-    <row r="249" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A249" s="8">
         <v>1696</v>
       </c>
@@ -23325,7 +23324,7 @@
       <c r="AD249" s="8"/>
       <c r="AE249" s="8"/>
     </row>
-    <row r="250" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A250" s="8">
         <v>1697</v>
       </c>
@@ -23396,7 +23395,7 @@
       <c r="AD250" s="8"/>
       <c r="AE250" s="8"/>
     </row>
-    <row r="251" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A251" s="8">
         <v>1698</v>
       </c>
@@ -23467,7 +23466,7 @@
       <c r="AD251" s="8"/>
       <c r="AE251" s="8"/>
     </row>
-    <row r="252" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A252" s="8">
         <v>1699</v>
       </c>
@@ -23538,7 +23537,7 @@
       <c r="AD252" s="8"/>
       <c r="AE252" s="8"/>
     </row>
-    <row r="253" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A253" s="8">
         <v>1700</v>
       </c>
@@ -23609,7 +23608,7 @@
       <c r="AD253" s="8"/>
       <c r="AE253" s="8"/>
     </row>
-    <row r="254" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A254" s="8">
         <v>1701</v>
       </c>
@@ -23680,7 +23679,7 @@
       <c r="AD254" s="8"/>
       <c r="AE254" s="8"/>
     </row>
-    <row r="255" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A255" s="8">
         <v>1707</v>
       </c>
@@ -23761,7 +23760,7 @@
       <c r="AD255" s="8"/>
       <c r="AE255" s="8"/>
     </row>
-    <row r="256" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A256" s="8">
         <v>1708</v>
       </c>
@@ -23842,7 +23841,7 @@
       <c r="AD256" s="8"/>
       <c r="AE256" s="8"/>
     </row>
-    <row r="257" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A257" s="8">
         <v>1709</v>
       </c>
@@ -23923,7 +23922,7 @@
       <c r="AD257" s="8"/>
       <c r="AE257" s="8"/>
     </row>
-    <row r="258" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A258" s="8">
         <v>1710</v>
       </c>
@@ -24004,7 +24003,7 @@
       <c r="AD258" s="8"/>
       <c r="AE258" s="8"/>
     </row>
-    <row r="259" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A259" s="8">
         <v>1711</v>
       </c>
@@ -24085,7 +24084,7 @@
       <c r="AD259" s="8"/>
       <c r="AE259" s="8"/>
     </row>
-    <row r="260" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A260" s="8">
         <v>1712</v>
       </c>
@@ -24166,7 +24165,7 @@
       <c r="AD260" s="8"/>
       <c r="AE260" s="8"/>
     </row>
-    <row r="261" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A261" s="8">
         <v>1713</v>
       </c>
@@ -24237,7 +24236,7 @@
       <c r="AD261" s="8"/>
       <c r="AE261" s="8"/>
     </row>
-    <row r="262" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A262" s="8">
         <v>1714</v>
       </c>
@@ -24310,7 +24309,7 @@
       <c r="AD262" s="8"/>
       <c r="AE262" s="8"/>
     </row>
-    <row r="263" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A263" s="8">
         <v>1715</v>
       </c>
@@ -24383,7 +24382,7 @@
       <c r="AD263" s="8"/>
       <c r="AE263" s="8"/>
     </row>
-    <row r="264" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A264" s="8">
         <v>1716</v>
       </c>
@@ -24456,7 +24455,7 @@
       <c r="AD264" s="8"/>
       <c r="AE264" s="8"/>
     </row>
-    <row r="265" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A265" s="8">
         <v>1717</v>
       </c>
@@ -24529,7 +24528,7 @@
       <c r="AD265" s="8"/>
       <c r="AE265" s="8"/>
     </row>
-    <row r="266" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A266" s="8">
         <v>1718</v>
       </c>
@@ -24602,7 +24601,7 @@
       <c r="AD266" s="8"/>
       <c r="AE266" s="8"/>
     </row>
-    <row r="267" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A267" s="8">
         <v>1719</v>
       </c>
@@ -24681,7 +24680,7 @@
       <c r="AD267" s="8"/>
       <c r="AE267" s="8"/>
     </row>
-    <row r="268" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A268" s="8">
         <v>1720</v>
       </c>
@@ -24760,7 +24759,7 @@
       <c r="AD268" s="8"/>
       <c r="AE268" s="8"/>
     </row>
-    <row r="269" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A269" s="8">
         <v>1721</v>
       </c>
@@ -24839,7 +24838,7 @@
       <c r="AD269" s="8"/>
       <c r="AE269" s="8"/>
     </row>
-    <row r="270" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A270" s="8">
         <v>1722</v>
       </c>
@@ -24920,7 +24919,7 @@
       <c r="AD270" s="8"/>
       <c r="AE270" s="8"/>
     </row>
-    <row r="271" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A271" s="8">
         <v>1723</v>
       </c>
@@ -24999,7 +24998,7 @@
       <c r="AD271" s="8"/>
       <c r="AE271" s="8"/>
     </row>
-    <row r="272" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A272" s="8">
         <v>1724</v>
       </c>
@@ -25080,7 +25079,7 @@
       <c r="AD272" s="8"/>
       <c r="AE272" s="8"/>
     </row>
-    <row r="273" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A273" s="8">
         <v>1725</v>
       </c>
@@ -25153,7 +25152,7 @@
       <c r="AD273" s="8"/>
       <c r="AE273" s="8"/>
     </row>
-    <row r="274" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A274" s="8">
         <v>1726</v>
       </c>
@@ -25226,7 +25225,7 @@
       <c r="AD274" s="8"/>
       <c r="AE274" s="8"/>
     </row>
-    <row r="275" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A275" s="8">
         <v>1727</v>
       </c>
@@ -25299,7 +25298,7 @@
       <c r="AD275" s="8"/>
       <c r="AE275" s="8"/>
     </row>
-    <row r="276" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A276" s="8">
         <v>1728</v>
       </c>
@@ -25372,7 +25371,7 @@
       <c r="AD276" s="8"/>
       <c r="AE276" s="8"/>
     </row>
-    <row r="277" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A277" s="8">
         <v>1729</v>
       </c>
@@ -25445,7 +25444,7 @@
       <c r="AD277" s="8"/>
       <c r="AE277" s="8"/>
     </row>
-    <row r="278" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A278" s="8">
         <v>1730</v>
       </c>
@@ -25518,7 +25517,7 @@
       <c r="AD278" s="8"/>
       <c r="AE278" s="8"/>
     </row>
-    <row r="279" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A279" s="8">
         <v>1731</v>
       </c>
@@ -25589,7 +25588,7 @@
       <c r="AD279" s="8"/>
       <c r="AE279" s="8"/>
     </row>
-    <row r="280" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A280" s="8">
         <v>1732</v>
       </c>
@@ -25662,7 +25661,7 @@
       <c r="AD280" s="8"/>
       <c r="AE280" s="8"/>
     </row>
-    <row r="281" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A281" s="8">
         <v>1733</v>
       </c>
@@ -25733,7 +25732,7 @@
       <c r="AD281" s="8"/>
       <c r="AE281" s="8"/>
     </row>
-    <row r="282" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A282" s="8">
         <v>1734</v>
       </c>
@@ -25802,7 +25801,7 @@
       <c r="AD282" s="8"/>
       <c r="AE282" s="8"/>
     </row>
-    <row r="283" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A283" s="8">
         <v>1735</v>
       </c>
@@ -25875,7 +25874,7 @@
       <c r="AD283" s="8"/>
       <c r="AE283" s="8"/>
     </row>
-    <row r="284" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A284" s="8">
         <v>1736</v>
       </c>
@@ -25946,7 +25945,7 @@
       <c r="AD284" s="8"/>
       <c r="AE284" s="8"/>
     </row>
-    <row r="285" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A285" s="8">
         <v>1737</v>
       </c>
@@ -26017,7 +26016,7 @@
       <c r="AD285" s="8"/>
       <c r="AE285" s="8"/>
     </row>
-    <row r="286" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A286" s="8">
         <v>1738</v>
       </c>
@@ -26090,7 +26089,7 @@
       <c r="AD286" s="8"/>
       <c r="AE286" s="8"/>
     </row>
-    <row r="287" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A287" s="8">
         <v>1739</v>
       </c>
@@ -26159,7 +26158,7 @@
       <c r="AD287" s="8"/>
       <c r="AE287" s="8"/>
     </row>
-    <row r="288" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A288" s="8">
         <v>1740</v>
       </c>
@@ -26232,7 +26231,7 @@
       <c r="AD288" s="8"/>
       <c r="AE288" s="8"/>
     </row>
-    <row r="289" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A289" s="8">
         <v>1741</v>
       </c>
@@ -26301,7 +26300,7 @@
       <c r="AD289" s="8"/>
       <c r="AE289" s="8"/>
     </row>
-    <row r="290" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A290" s="8">
         <v>1742</v>
       </c>
@@ -26370,7 +26369,7 @@
       <c r="AD290" s="8"/>
       <c r="AE290" s="8"/>
     </row>
-    <row r="291" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A291" s="8">
         <v>1743</v>
       </c>
@@ -26443,7 +26442,7 @@
       <c r="AD291" s="8"/>
       <c r="AE291" s="8"/>
     </row>
-    <row r="292" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A292" s="8">
         <v>1744</v>
       </c>
@@ -26514,7 +26513,7 @@
       <c r="AD292" s="8"/>
       <c r="AE292" s="8"/>
     </row>
-    <row r="293" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A293" s="8">
         <v>1745</v>
       </c>
@@ -26583,7 +26582,7 @@
       <c r="AD293" s="8"/>
       <c r="AE293" s="8"/>
     </row>
-    <row r="294" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A294" s="8">
         <v>1746</v>
       </c>
@@ -26664,7 +26663,7 @@
       <c r="AD294" s="8"/>
       <c r="AE294" s="8"/>
     </row>
-    <row r="295" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A295" s="8">
         <v>1747</v>
       </c>
@@ -26745,7 +26744,7 @@
       <c r="AD295" s="8"/>
       <c r="AE295" s="8"/>
     </row>
-    <row r="296" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A296" s="8">
         <v>1748</v>
       </c>
@@ -26826,7 +26825,7 @@
       <c r="AD296" s="8"/>
       <c r="AE296" s="8"/>
     </row>
-    <row r="297" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A297" s="8">
         <v>1749</v>
       </c>
@@ -26907,7 +26906,7 @@
       <c r="AD297" s="8"/>
       <c r="AE297" s="8"/>
     </row>
-    <row r="298" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A298" s="8">
         <v>1750</v>
       </c>
@@ -26988,7 +26987,7 @@
       <c r="AD298" s="8"/>
       <c r="AE298" s="8"/>
     </row>
-    <row r="299" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A299" s="8">
         <v>1752</v>
       </c>
@@ -27069,7 +27068,7 @@
       <c r="AD299" s="8"/>
       <c r="AE299" s="8"/>
     </row>
-    <row r="300" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A300" s="8">
         <v>1753</v>
       </c>
@@ -27150,7 +27149,7 @@
       <c r="AD300" s="8"/>
       <c r="AE300" s="8"/>
     </row>
-    <row r="301" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A301" s="8">
         <v>1754</v>
       </c>
@@ -27231,7 +27230,7 @@
       <c r="AD301" s="8"/>
       <c r="AE301" s="8"/>
     </row>
-    <row r="302" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A302" s="8">
         <v>1755</v>
       </c>
@@ -27312,7 +27311,7 @@
       <c r="AD302" s="8"/>
       <c r="AE302" s="8"/>
     </row>
-    <row r="303" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A303" s="8">
         <v>1756</v>
       </c>
@@ -27393,7 +27392,7 @@
       <c r="AD303" s="8"/>
       <c r="AE303" s="8"/>
     </row>
-    <row r="304" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A304" s="8">
         <v>1759</v>
       </c>
@@ -27464,7 +27463,7 @@
       <c r="AD304" s="8"/>
       <c r="AE304" s="8"/>
     </row>
-    <row r="305" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A305" s="8">
         <v>1760</v>
       </c>
@@ -27535,7 +27534,7 @@
       <c r="AD305" s="8"/>
       <c r="AE305" s="8"/>
     </row>
-    <row r="306" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A306" s="8">
         <v>1762</v>
       </c>
@@ -27606,7 +27605,7 @@
       <c r="AD306" s="8"/>
       <c r="AE306" s="8"/>
     </row>
-    <row r="307" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A307" s="8">
         <v>1763</v>
       </c>
@@ -27679,7 +27678,7 @@
       <c r="AD307" s="8"/>
       <c r="AE307" s="8"/>
     </row>
-    <row r="308" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A308" s="8">
         <v>1764</v>
       </c>
@@ -27750,7 +27749,7 @@
       <c r="AD308" s="8"/>
       <c r="AE308" s="8"/>
     </row>
-    <row r="309" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A309" s="8">
         <v>1767</v>
       </c>
@@ -27821,7 +27820,7 @@
       <c r="AD309" s="8"/>
       <c r="AE309" s="8"/>
     </row>
-    <row r="310" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A310" s="8">
         <v>1768</v>
       </c>
@@ -27892,7 +27891,7 @@
       <c r="AD310" s="8"/>
       <c r="AE310" s="8"/>
     </row>
-    <row r="311" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A311" s="8">
         <v>1769</v>
       </c>
@@ -27963,7 +27962,7 @@
       <c r="AD311" s="8"/>
       <c r="AE311" s="8"/>
     </row>
-    <row r="312" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A312" s="8">
         <v>1770</v>
       </c>
@@ -28034,7 +28033,7 @@
       <c r="AD312" s="8"/>
       <c r="AE312" s="8"/>
     </row>
-    <row r="313" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A313" s="8">
         <v>1771</v>
       </c>
@@ -28415,7 +28414,7 @@
       <c r="AD317" s="8"/>
       <c r="AE317" s="8"/>
     </row>
-    <row r="318" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A318" s="8">
         <v>1776</v>
       </c>
@@ -28486,7 +28485,7 @@
       <c r="AD318" s="8"/>
       <c r="AE318" s="8"/>
     </row>
-    <row r="319" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A319" s="8">
         <v>1777</v>
       </c>
@@ -28557,7 +28556,7 @@
       <c r="AD319" s="8"/>
       <c r="AE319" s="8"/>
     </row>
-    <row r="320" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A320" s="8">
         <v>1778</v>
       </c>
@@ -28628,7 +28627,7 @@
       <c r="AD320" s="8"/>
       <c r="AE320" s="8"/>
     </row>
-    <row r="321" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A321" s="8">
         <v>1779</v>
       </c>
@@ -28699,7 +28698,7 @@
       <c r="AD321" s="8"/>
       <c r="AE321" s="8"/>
     </row>
-    <row r="322" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A322" s="8">
         <v>1780</v>
       </c>
@@ -28768,7 +28767,7 @@
       <c r="AD322" s="8"/>
       <c r="AE322" s="8"/>
     </row>
-    <row r="323" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A323" s="8">
         <v>1781</v>
       </c>
@@ -28837,7 +28836,7 @@
       <c r="AD323" s="8"/>
       <c r="AE323" s="8"/>
     </row>
-    <row r="324" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A324" s="8">
         <v>1782</v>
       </c>
@@ -28904,7 +28903,7 @@
       <c r="AD324" s="8"/>
       <c r="AE324" s="8"/>
     </row>
-    <row r="325" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A325" s="8">
         <v>1783</v>
       </c>
@@ -28973,7 +28972,7 @@
       <c r="AD325" s="8"/>
       <c r="AE325" s="8"/>
     </row>
-    <row r="326" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A326" s="8">
         <v>1784</v>
       </c>
@@ -29040,7 +29039,7 @@
       <c r="AD326" s="8"/>
       <c r="AE326" s="8"/>
     </row>
-    <row r="327" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A327" s="8">
         <v>1785</v>
       </c>
@@ -29107,7 +29106,7 @@
       <c r="AD327" s="8"/>
       <c r="AE327" s="8"/>
     </row>
-    <row r="328" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A328" s="8">
         <v>1792</v>
       </c>
@@ -29174,7 +29173,7 @@
       <c r="AD328" s="8"/>
       <c r="AE328" s="8"/>
     </row>
-    <row r="329" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A329" s="8">
         <v>1793</v>
       </c>
@@ -29241,7 +29240,7 @@
       <c r="AD329" s="8"/>
       <c r="AE329" s="8"/>
     </row>
-    <row r="330" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A330" s="8">
         <v>1794</v>
       </c>
@@ -29308,7 +29307,7 @@
       <c r="AD330" s="8"/>
       <c r="AE330" s="8"/>
     </row>
-    <row r="331" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A331" s="8">
         <v>1795</v>
       </c>
@@ -29379,7 +29378,7 @@
       <c r="AD331" s="8"/>
       <c r="AE331" s="8"/>
     </row>
-    <row r="332" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A332" s="8">
         <v>1796</v>
       </c>
@@ -29450,7 +29449,7 @@
       <c r="AD332" s="8"/>
       <c r="AE332" s="8"/>
     </row>
-    <row r="333" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A333" s="8">
         <v>1797</v>
       </c>
@@ -29521,7 +29520,7 @@
       <c r="AD333" s="8"/>
       <c r="AE333" s="8"/>
     </row>
-    <row r="334" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A334" s="8">
         <v>1798</v>
       </c>
@@ -29594,7 +29593,7 @@
       <c r="AD334" s="8"/>
       <c r="AE334" s="8"/>
     </row>
-    <row r="335" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A335" s="8">
         <v>1799</v>
       </c>
@@ -29665,7 +29664,7 @@
       <c r="AD335" s="8"/>
       <c r="AE335" s="8"/>
     </row>
-    <row r="336" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A336" s="8">
         <v>1800</v>
       </c>
@@ -29734,7 +29733,7 @@
       <c r="AD336" s="8"/>
       <c r="AE336" s="8"/>
     </row>
-    <row r="337" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A337" s="8">
         <v>1801</v>
       </c>
@@ -29801,7 +29800,7 @@
       <c r="AD337" s="8"/>
       <c r="AE337" s="8"/>
     </row>
-    <row r="338" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A338" s="8">
         <v>1811</v>
       </c>
@@ -29872,7 +29871,7 @@
       <c r="AD338" s="8"/>
       <c r="AE338" s="8"/>
     </row>
-    <row r="339" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A339" s="8">
         <v>1812</v>
       </c>
@@ -29943,7 +29942,7 @@
       <c r="AD339" s="8"/>
       <c r="AE339" s="8"/>
     </row>
-    <row r="340" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A340" s="8">
         <v>1813</v>
       </c>
@@ -30012,7 +30011,7 @@
       <c r="AD340" s="8"/>
       <c r="AE340" s="8"/>
     </row>
-    <row r="341" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A341" s="8">
         <v>1814</v>
       </c>
@@ -30085,7 +30084,7 @@
       <c r="AD341" s="8"/>
       <c r="AE341" s="8"/>
     </row>
-    <row r="342" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A342" s="8">
         <v>1815</v>
       </c>
@@ -30158,7 +30157,7 @@
       <c r="AD342" s="8"/>
       <c r="AE342" s="8"/>
     </row>
-    <row r="343" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A343" s="8">
         <v>1816</v>
       </c>
@@ -30231,7 +30230,7 @@
       <c r="AD343" s="8"/>
       <c r="AE343" s="8"/>
     </row>
-    <row r="344" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A344" s="8">
         <v>1817</v>
       </c>
@@ -30302,7 +30301,7 @@
       <c r="AD344" s="8"/>
       <c r="AE344" s="8"/>
     </row>
-    <row r="345" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A345" s="8">
         <v>1818</v>
       </c>
@@ -30375,7 +30374,7 @@
       <c r="AD345" s="8"/>
       <c r="AE345" s="8"/>
     </row>
-    <row r="346" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A346" s="8">
         <v>1819</v>
       </c>
@@ -30446,7 +30445,7 @@
       <c r="AD346" s="8"/>
       <c r="AE346" s="8"/>
     </row>
-    <row r="347" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A347" s="8">
         <v>1820</v>
       </c>
@@ -30517,7 +30516,7 @@
       <c r="AD347" s="8"/>
       <c r="AE347" s="8"/>
     </row>
-    <row r="348" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A348" s="8">
         <v>1821</v>
       </c>
@@ -30588,7 +30587,7 @@
       <c r="AD348" s="8"/>
       <c r="AE348" s="8"/>
     </row>
-    <row r="349" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A349" s="8">
         <v>1822</v>
       </c>
@@ -30661,7 +30660,7 @@
       <c r="AD349" s="8"/>
       <c r="AE349" s="8"/>
     </row>
-    <row r="350" spans="1:31" ht="302.39999999999998" hidden="1" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:31" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A350" s="8">
         <v>1823</v>
       </c>
@@ -30732,7 +30731,7 @@
       <c r="AD350" s="8"/>
       <c r="AE350" s="8"/>
     </row>
-    <row r="351" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A351" s="8">
         <v>1824</v>
       </c>
@@ -30803,7 +30802,7 @@
       <c r="AD351" s="8"/>
       <c r="AE351" s="8"/>
     </row>
-    <row r="352" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A352" s="8">
         <v>1825</v>
       </c>
@@ -30876,7 +30875,7 @@
       <c r="AD352" s="8"/>
       <c r="AE352" s="8"/>
     </row>
-    <row r="353" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A353" s="8">
         <v>1826</v>
       </c>
@@ -30947,7 +30946,7 @@
       <c r="AD353" s="8"/>
       <c r="AE353" s="8"/>
     </row>
-    <row r="354" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A354" s="8">
         <v>1827</v>
       </c>
@@ -31016,7 +31015,7 @@
       <c r="AD354" s="8"/>
       <c r="AE354" s="8"/>
     </row>
-    <row r="355" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A355" s="8">
         <v>1828</v>
       </c>
@@ -31085,7 +31084,7 @@
       <c r="AD355" s="8"/>
       <c r="AE355" s="8"/>
     </row>
-    <row r="356" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A356" s="8">
         <v>1829</v>
       </c>
@@ -31154,7 +31153,7 @@
       <c r="AD356" s="8"/>
       <c r="AE356" s="8"/>
     </row>
-    <row r="357" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A357" s="8">
         <v>1830</v>
       </c>
@@ -31223,7 +31222,7 @@
       <c r="AD357" s="8"/>
       <c r="AE357" s="8"/>
     </row>
-    <row r="358" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A358" s="8">
         <v>1831</v>
       </c>
@@ -31294,7 +31293,7 @@
       <c r="AD358" s="8"/>
       <c r="AE358" s="8"/>
     </row>
-    <row r="359" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A359" s="8">
         <v>1832</v>
       </c>
@@ -31365,7 +31364,7 @@
       <c r="AD359" s="8"/>
       <c r="AE359" s="8"/>
     </row>
-    <row r="360" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A360" s="8">
         <v>1833</v>
       </c>
@@ -31436,7 +31435,7 @@
       <c r="AD360" s="8"/>
       <c r="AE360" s="8"/>
     </row>
-    <row r="361" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A361" s="8">
         <v>1834</v>
       </c>
@@ -31507,7 +31506,7 @@
       <c r="AD361" s="8"/>
       <c r="AE361" s="8"/>
     </row>
-    <row r="362" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A362" s="8">
         <v>1835</v>
       </c>
@@ -31578,7 +31577,7 @@
       <c r="AD362" s="8"/>
       <c r="AE362" s="8"/>
     </row>
-    <row r="363" spans="1:31" ht="388.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:31" ht="388.8" x14ac:dyDescent="0.3">
       <c r="A363" s="8">
         <v>1836</v>
       </c>
@@ -31649,7 +31648,7 @@
       <c r="AD363" s="8"/>
       <c r="AE363" s="8"/>
     </row>
-    <row r="364" spans="1:31" ht="388.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:31" ht="388.8" x14ac:dyDescent="0.3">
       <c r="A364" s="8">
         <v>1837</v>
       </c>
@@ -31720,7 +31719,7 @@
       <c r="AD364" s="8"/>
       <c r="AE364" s="8"/>
     </row>
-    <row r="365" spans="1:31" ht="388.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:31" ht="388.8" x14ac:dyDescent="0.3">
       <c r="A365" s="8">
         <v>1838</v>
       </c>
@@ -31791,7 +31790,7 @@
       <c r="AD365" s="8"/>
       <c r="AE365" s="8"/>
     </row>
-    <row r="366" spans="1:31" ht="388.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:31" ht="388.8" x14ac:dyDescent="0.3">
       <c r="A366" s="8">
         <v>1839</v>
       </c>
@@ -31862,7 +31861,7 @@
       <c r="AD366" s="8"/>
       <c r="AE366" s="8"/>
     </row>
-    <row r="367" spans="1:31" ht="388.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:31" ht="388.8" x14ac:dyDescent="0.3">
       <c r="A367" s="8">
         <v>1840</v>
       </c>
@@ -31933,7 +31932,7 @@
       <c r="AD367" s="8"/>
       <c r="AE367" s="8"/>
     </row>
-    <row r="368" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A368" s="8">
         <v>1841</v>
       </c>
@@ -32006,7 +32005,7 @@
       <c r="AD368" s="8"/>
       <c r="AE368" s="8"/>
     </row>
-    <row r="369" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A369" s="8">
         <v>1842</v>
       </c>
@@ -32075,7 +32074,7 @@
       <c r="AD369" s="8"/>
       <c r="AE369" s="8"/>
     </row>
-    <row r="370" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A370" s="8">
         <v>1843</v>
       </c>
@@ -32146,7 +32145,7 @@
       <c r="AD370" s="8"/>
       <c r="AE370" s="8"/>
     </row>
-    <row r="371" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A371" s="8">
         <v>1844</v>
       </c>
@@ -32215,7 +32214,7 @@
       <c r="AD371" s="8"/>
       <c r="AE371" s="8"/>
     </row>
-    <row r="372" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A372" s="8">
         <v>1845</v>
       </c>
@@ -32284,7 +32283,7 @@
       <c r="AD372" s="8"/>
       <c r="AE372" s="8"/>
     </row>
-    <row r="373" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A373" s="8">
         <v>1846</v>
       </c>
@@ -32353,7 +32352,7 @@
       <c r="AD373" s="8"/>
       <c r="AE373" s="8"/>
     </row>
-    <row r="374" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A374" s="8">
         <v>1847</v>
       </c>
@@ -32426,7 +32425,7 @@
       <c r="AD374" s="8"/>
       <c r="AE374" s="8"/>
     </row>
-    <row r="375" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A375" s="8">
         <v>1848</v>
       </c>
@@ -32499,7 +32498,7 @@
       <c r="AD375" s="8"/>
       <c r="AE375" s="8"/>
     </row>
-    <row r="376" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A376" s="8">
         <v>1849</v>
       </c>
@@ -32568,7 +32567,7 @@
       <c r="AD376" s="8"/>
       <c r="AE376" s="8"/>
     </row>
-    <row r="377" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A377" s="8">
         <v>1850</v>
       </c>
@@ -32641,7 +32640,7 @@
       <c r="AD377" s="8"/>
       <c r="AE377" s="8"/>
     </row>
-    <row r="378" spans="1:31" ht="360" hidden="1" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:31" ht="360" x14ac:dyDescent="0.3">
       <c r="A378" s="8">
         <v>1851</v>
       </c>
@@ -32710,7 +32709,7 @@
       <c r="AD378" s="8"/>
       <c r="AE378" s="8"/>
     </row>
-    <row r="379" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A379" s="8">
         <v>1852</v>
       </c>
@@ -32785,7 +32784,7 @@
       <c r="AD379" s="8"/>
       <c r="AE379" s="8"/>
     </row>
-    <row r="380" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A380" s="8">
         <v>1853</v>
       </c>
@@ -32856,7 +32855,7 @@
       <c r="AD380" s="8"/>
       <c r="AE380" s="8"/>
     </row>
-    <row r="381" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A381" s="8">
         <v>1854</v>
       </c>
@@ -32925,7 +32924,7 @@
       <c r="AD381" s="8"/>
       <c r="AE381" s="8"/>
     </row>
-    <row r="382" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A382" s="8">
         <v>1855</v>
       </c>
@@ -32994,7 +32993,7 @@
       <c r="AD382" s="8"/>
       <c r="AE382" s="8"/>
     </row>
-    <row r="383" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A383" s="8">
         <v>1856</v>
       </c>
@@ -33065,7 +33064,7 @@
       <c r="AD383" s="8"/>
       <c r="AE383" s="8"/>
     </row>
-    <row r="384" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A384" s="8">
         <v>1857</v>
       </c>
@@ -33138,7 +33137,7 @@
       <c r="AD384" s="8"/>
       <c r="AE384" s="8"/>
     </row>
-    <row r="385" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A385" s="8">
         <v>1858</v>
       </c>
@@ -33211,7 +33210,7 @@
       <c r="AD385" s="8"/>
       <c r="AE385" s="8"/>
     </row>
-    <row r="386" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A386" s="8">
         <v>1859</v>
       </c>
@@ -33282,7 +33281,7 @@
       <c r="AD386" s="8"/>
       <c r="AE386" s="8"/>
     </row>
-    <row r="387" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A387" s="8">
         <v>1860</v>
       </c>
@@ -33353,7 +33352,7 @@
       <c r="AD387" s="8"/>
       <c r="AE387" s="8"/>
     </row>
-    <row r="388" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A388" s="8">
         <v>1862</v>
       </c>
@@ -33420,7 +33419,7 @@
       <c r="AD388" s="8"/>
       <c r="AE388" s="8"/>
     </row>
-    <row r="389" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A389" s="8">
         <v>1863</v>
       </c>
@@ -33487,7 +33486,7 @@
       <c r="AD389" s="8"/>
       <c r="AE389" s="8"/>
     </row>
-    <row r="390" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A390" s="8">
         <v>1864</v>
       </c>
@@ -33554,7 +33553,7 @@
       <c r="AD390" s="8"/>
       <c r="AE390" s="8"/>
     </row>
-    <row r="391" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A391" s="8">
         <v>1866</v>
       </c>
@@ -33625,7 +33624,7 @@
       <c r="AD391" s="8"/>
       <c r="AE391" s="8"/>
     </row>
-    <row r="392" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A392" s="8">
         <v>1867</v>
       </c>
@@ -33696,7 +33695,7 @@
       <c r="AD392" s="8"/>
       <c r="AE392" s="8"/>
     </row>
-    <row r="393" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A393" s="8">
         <v>1868</v>
       </c>
@@ -33767,7 +33766,7 @@
       <c r="AD393" s="8"/>
       <c r="AE393" s="8"/>
     </row>
-    <row r="394" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A394" s="8">
         <v>1869</v>
       </c>
@@ -33834,7 +33833,7 @@
       <c r="AD394" s="8"/>
       <c r="AE394" s="8"/>
     </row>
-    <row r="395" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A395" s="8">
         <v>1870</v>
       </c>
@@ -33901,7 +33900,7 @@
       <c r="AD395" s="8"/>
       <c r="AE395" s="8"/>
     </row>
-    <row r="396" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A396" s="8">
         <v>1872</v>
       </c>
@@ -33972,7 +33971,7 @@
       <c r="AD396" s="8"/>
       <c r="AE396" s="8"/>
     </row>
-    <row r="397" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A397" s="8">
         <v>1873</v>
       </c>
@@ -34043,7 +34042,7 @@
       <c r="AD397" s="8"/>
       <c r="AE397" s="8"/>
     </row>
-    <row r="398" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A398" s="8">
         <v>1874</v>
       </c>
@@ -34110,7 +34109,7 @@
       <c r="AD398" s="8"/>
       <c r="AE398" s="8"/>
     </row>
-    <row r="399" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A399" s="8">
         <v>1875</v>
       </c>
@@ -34177,7 +34176,7 @@
       <c r="AD399" s="8"/>
       <c r="AE399" s="8"/>
     </row>
-    <row r="400" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A400" s="8">
         <v>1876</v>
       </c>
@@ -34244,7 +34243,7 @@
       <c r="AD400" s="8"/>
       <c r="AE400" s="8"/>
     </row>
-    <row r="401" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A401" s="8">
         <v>1877</v>
       </c>
@@ -34311,7 +34310,7 @@
       <c r="AD401" s="8"/>
       <c r="AE401" s="8"/>
     </row>
-    <row r="402" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A402" s="8">
         <v>1878</v>
       </c>
@@ -34382,7 +34381,7 @@
       <c r="AD402" s="8"/>
       <c r="AE402" s="8"/>
     </row>
-    <row r="403" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A403" s="8">
         <v>1879</v>
       </c>
@@ -34453,7 +34452,7 @@
       <c r="AD403" s="8"/>
       <c r="AE403" s="8"/>
     </row>
-    <row r="404" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A404" s="8">
         <v>1880</v>
       </c>
@@ -34520,7 +34519,7 @@
       <c r="AD404" s="8"/>
       <c r="AE404" s="8"/>
     </row>
-    <row r="405" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A405" s="8">
         <v>1881</v>
       </c>
@@ -34587,7 +34586,7 @@
       <c r="AD405" s="8"/>
       <c r="AE405" s="8"/>
     </row>
-    <row r="406" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A406" s="8">
         <v>1882</v>
       </c>
@@ -34654,7 +34653,7 @@
       <c r="AD406" s="8"/>
       <c r="AE406" s="8"/>
     </row>
-    <row r="407" spans="1:31" ht="230.4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:31" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A407" s="8">
         <v>1883</v>
       </c>
@@ -34721,7 +34720,7 @@
       <c r="AD407" s="8"/>
       <c r="AE407" s="8"/>
     </row>
-    <row r="408" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A408" s="8">
         <v>1885</v>
       </c>
@@ -34790,7 +34789,7 @@
       <c r="AD408" s="8"/>
       <c r="AE408" s="8"/>
     </row>
-    <row r="409" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A409" s="8">
         <v>1886</v>
       </c>
@@ -34859,7 +34858,7 @@
       <c r="AD409" s="8"/>
       <c r="AE409" s="8"/>
     </row>
-    <row r="410" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A410" s="8">
         <v>1887</v>
       </c>
@@ -34928,7 +34927,7 @@
       <c r="AD410" s="8"/>
       <c r="AE410" s="8"/>
     </row>
-    <row r="411" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A411" s="8">
         <v>1888</v>
       </c>
@@ -34997,7 +34996,7 @@
       <c r="AD411" s="8"/>
       <c r="AE411" s="8"/>
     </row>
-    <row r="412" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A412" s="8">
         <v>1889</v>
       </c>
@@ -35064,7 +35063,7 @@
       <c r="AD412" s="8"/>
       <c r="AE412" s="8"/>
     </row>
-    <row r="413" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A413" s="8">
         <v>1890</v>
       </c>
@@ -35133,7 +35132,7 @@
       <c r="AD413" s="8"/>
       <c r="AE413" s="8"/>
     </row>
-    <row r="414" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A414" s="8">
         <v>1891</v>
       </c>
@@ -35202,7 +35201,7 @@
       <c r="AD414" s="8"/>
       <c r="AE414" s="8"/>
     </row>
-    <row r="415" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A415" s="8">
         <v>1892</v>
       </c>
@@ -35271,7 +35270,7 @@
       <c r="AD415" s="8"/>
       <c r="AE415" s="8"/>
     </row>
-    <row r="416" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A416" s="8">
         <v>1893</v>
       </c>
@@ -35340,7 +35339,7 @@
       <c r="AD416" s="8"/>
       <c r="AE416" s="8"/>
     </row>
-    <row r="417" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A417" s="8">
         <v>1894</v>
       </c>
@@ -35407,7 +35406,7 @@
       <c r="AD417" s="8"/>
       <c r="AE417" s="8"/>
     </row>
-    <row r="418" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A418" s="8">
         <v>1895</v>
       </c>
@@ -35474,7 +35473,7 @@
       <c r="AD418" s="8"/>
       <c r="AE418" s="8"/>
     </row>
-    <row r="419" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A419" s="8">
         <v>1896</v>
       </c>
@@ -35541,7 +35540,7 @@
       <c r="AD419" s="8"/>
       <c r="AE419" s="8"/>
     </row>
-    <row r="420" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A420" s="8">
         <v>1897</v>
       </c>
@@ -35610,7 +35609,7 @@
       <c r="AD420" s="8"/>
       <c r="AE420" s="8"/>
     </row>
-    <row r="421" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A421" s="8">
         <v>1898</v>
       </c>
@@ -35679,7 +35678,7 @@
       <c r="AD421" s="8"/>
       <c r="AE421" s="8"/>
     </row>
-    <row r="422" spans="1:31" ht="409.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:31" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A422" s="3">
         <v>1899</v>
       </c>
@@ -35750,13 +35749,6 @@
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <autoFilter ref="A1:AE422" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="440"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>